<commit_message>
docs: parts list without 48 V / 24 V supplies (in stock)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parts-list.xlsx
+++ b/docs/parts-list.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -484,7 +484,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bump'em parts list (everything except motor and encoder)</t>
+          <t>Bump'em parts list (everything except motor, encoder, 48 V and 24 V supplies)</t>
         </is>
       </c>
     </row>
@@ -664,12 +664,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>48 V supply</t>
+          <t>AC power cord for the 48 V supply</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mean Well RSP-2000-48</t>
+          <t>fitted by the electrician</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -680,24 +680,14 @@
           <t>tower</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n">
-        <v>365.2</v>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Reichelt, incl. 19 % VAT</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>https://www.reichelt.com/de/en/shop/product/switching_power_supply_pfc_2016_w_48_v_42_a-147912</t>
-        </is>
-      </c>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>to check</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" s="5">
         <f>IF(F8="","",D8*F8*IF(E8="tower",$C$3,1))</f>
         <v/>
@@ -711,12 +701,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AC power cord for the 48 V supply</t>
+          <t>E-stop connector for CN501</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>fitted by the electrician</t>
+          <t>Hirose DF11-12DS housing + DF11 crimp terminals</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -748,16 +738,16 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>E-stop connector for CN501</t>
+          <t>Ring terminals (supply +V / -V / earth)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hirose DF11-12DS housing + DF11 crimp terminals</t>
+          <t>for 14 AWG</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -785,16 +775,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ring terminals (supply +V / -V / earth)</t>
+          <t>Power cable chopper -&gt; ESCON J1 (m)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>for 14 AWG</t>
+          <t>14 AWG, 2-wire</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -817,17 +807,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Drive electronics</t>
+          <t>Force sensing</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Power cable chopper -&gt; ESCON J1 (m)</t>
+          <t>Load cell</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>14 AWG, 2-wire</t>
+          <t>DYMH-103, 100 kg</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -838,14 +828,24 @@
           <t>tower</t>
         </is>
       </c>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>to check</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="F12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>USD 60-130 (AliExpress / eBay), no EUR price found</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>https://www.daysensor.com/dymh-103/</t>
+        </is>
+      </c>
       <c r="J12" s="5">
         <f>IF(F12="","",D12*F12*IF(E12="tower",$C$3,1))</f>
         <v/>
@@ -859,12 +859,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Load cell</t>
+          <t>Load-cell amplifier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DYMH-103, 100 kg</t>
+          <t>Futek IAA100 (FSH03863)</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -876,21 +876,21 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>estimate</t>
+        <v>871</v>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>found</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>USD 60-130 (AliExpress / eBay), no EUR price found</t>
+          <t>Elkome (EU)</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>https://www.daysensor.com/dymh-103/</t>
+          <t>https://shop.elkome.com/en/iaa100-fsh03863-load-cell-amplifier</t>
         </is>
       </c>
       <c r="J13" s="5">
@@ -906,12 +906,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Load-cell amplifier</t>
+          <t>Ground distributor</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Futek IAA100 (FSH03863)</t>
+          <t>small screw terminal strip</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -922,24 +922,14 @@
           <t>tower</t>
         </is>
       </c>
-      <c r="F14" s="5" t="n">
-        <v>871</v>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Elkome (EU)</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="inlineStr">
-        <is>
-          <t>https://shop.elkome.com/en/iaa100-fsh03863-load-cell-amplifier</t>
-        </is>
-      </c>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>to check</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
       <c r="J14" s="5">
         <f>IF(F14="","",D14*F14*IF(E14="tower",$C$3,1))</f>
         <v/>
@@ -953,40 +943,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>24 V supply for the amplifier</t>
+          <t>Signal cable to the control board (m)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mean Well RS-15-24</t>
+          <t>multi-core, 7 wires</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>tower</t>
         </is>
       </c>
-      <c r="F15" s="5" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Reichelt, incl. 19 % VAT</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="inlineStr">
-        <is>
-          <t>https://www.reichelt.com/de/en/shop/product/switching_power_supply_15_w_0_62_a_24_v-137083</t>
-        </is>
-      </c>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>to check</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" s="5">
         <f>IF(F15="","",D15*F15*IF(E15="tower",$C$3,1))</f>
         <v/>
@@ -995,17 +975,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Force sensing</t>
+          <t>Mechanics (Stanford guide p. 11-13)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ground distributor</t>
+          <t>3D-printed motor mount, reel drum, drum cover</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>small screw terminal strip</t>
+          <t>PLA; drum 8 shells, &gt;= 70 % infill</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1022,7 +1002,11 @@
           <t>to check</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>printed in-house (filament below)</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" s="5">
         <f>IF(F16="","",D16*F16*IF(E16="tower",$C$3,1))</f>
@@ -1032,19 +1016,15 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Force sensing</t>
+          <t>Mechanics (Stanford guide p. 11-13)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Signal cable to the control board (m)</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>multi-core, 7 wires</t>
-        </is>
-      </c>
+          <t>Socket bolts #6-32 x 1/2 in</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="n">
         <v>3</v>
       </c>
@@ -1059,8 +1039,16 @@
           <t>to check</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>see Stanford BOM</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>https://biomechatronics.stanford.edu/bump-em</t>
+        </is>
+      </c>
       <c r="J17" s="5">
         <f>IF(F17="","",D17*F17*IF(E17="tower",$C$3,1))</f>
         <v/>
@@ -1074,16 +1062,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>3D-printed motor mount, reel drum, drum cover</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>PLA; drum 8 shells, &gt;= 70 % infill</t>
-        </is>
-      </c>
+          <t>Washers #6</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1098,10 +1082,14 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>printed in-house (filament below)</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
+          <t>see Stanford BOM</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>https://biomechatronics.stanford.edu/bump-em</t>
+        </is>
+      </c>
       <c r="J18" s="5">
         <f>IF(F18="","",D18*F18*IF(E18="tower",$C$3,1))</f>
         <v/>
@@ -1115,12 +1103,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Socket bolts #6-32 x 1/2 in</t>
+          <t>Flanged shaft collar</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1156,7 +1144,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Washers #6</t>
+          <t>Socket bolts M5 x 12 mm</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1174,16 +1162,8 @@
           <t>to check</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>see Stanford BOM</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>https://biomechatronics.stanford.edu/bump-em</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
       <c r="J20" s="5">
         <f>IF(F20="","",D20*F20*IF(E20="tower",$C$3,1))</f>
         <v/>
@@ -1197,12 +1177,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Flanged shaft collar</t>
+          <t>Washers M5</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1215,16 +1195,8 @@
           <t>to check</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>see Stanford BOM</t>
-        </is>
-      </c>
-      <c r="I21" s="7" t="inlineStr">
-        <is>
-          <t>https://biomechatronics.stanford.edu/bump-em</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" s="5">
         <f>IF(F21="","",D21*F21*IF(E21="tower",$C$3,1))</f>
         <v/>
@@ -1238,12 +1210,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Socket bolts M5 x 12 mm</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>Spider shaft coupler set</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>10 mm hub + 3/8 in hub + spider</t>
+        </is>
+      </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1256,8 +1232,16 @@
           <t>to check</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>see Stanford BOM</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>https://biomechatronics.stanford.edu/bump-em</t>
+        </is>
+      </c>
       <c r="J22" s="5">
         <f>IF(F22="","",D22*F22*IF(E22="tower",$C$3,1))</f>
         <v/>
@@ -1271,12 +1255,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Washers M5</t>
+          <t>Flanged bearings</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1289,8 +1273,16 @@
           <t>to check</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>see Stanford BOM</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>https://biomechatronics.stanford.edu/bump-em</t>
+        </is>
+      </c>
       <c r="J23" s="5">
         <f>IF(F23="","",D23*F23*IF(E23="tower",$C$3,1))</f>
         <v/>
@@ -1304,14 +1296,10 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Spider shaft coupler set</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>10 mm hub + 3/8 in hub + spider</t>
-        </is>
-      </c>
+          <t>Linear shaft 3/8 in x 3 in</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
         <v>1</v>
       </c>
@@ -1349,12 +1337,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Flanged bearings</t>
+          <t>Eyebolt + 1/4 in-20 nut</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1390,12 +1378,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Linear shaft 3/8 in x 3 in</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+          <t>Rope (m)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>braided Kevlar or Dyneema, &gt;= ~2 kN, diameter to match eyebolt</t>
+        </is>
+      </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1408,16 +1400,8 @@
           <t>to check</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>see Stanford BOM</t>
-        </is>
-      </c>
-      <c r="I26" s="7" t="inlineStr">
-        <is>
-          <t>https://biomechatronics.stanford.edu/bump-em</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" s="5">
         <f>IF(F26="","",D26*F26*IF(E26="tower",$C$3,1))</f>
         <v/>
@@ -1426,37 +1410,43 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mechanics (Stanford guide p. 11-13)</t>
+          <t>Control (once)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Eyebolt + 1/4 in-20 nut</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t>Microcontroller</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Teensy 4.1</t>
+        </is>
+      </c>
       <c r="D27" t="n">
         <v>1</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>tower</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="8" t="inlineStr">
-        <is>
-          <t>to check</t>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>37.49</v>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>found</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>see Stanford BOM</t>
+          <t>Antratek, incl. VAT</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>https://biomechatronics.stanford.edu/bump-em</t>
+          <t>https://www.antratek.de/teensy-4-1</t>
         </is>
       </c>
       <c r="J27" s="5">
@@ -1467,25 +1457,25 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mechanics (Stanford guide p. 11-13)</t>
+          <t>Control (once)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Rope (m)</t>
+          <t>Pin headers for the Teensy</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>braided Kevlar or Dyneema, &gt;= ~2 kN, diameter to match eyebolt</t>
+          <t>2.54 mm male, 2 x 24</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>tower</t>
+          <t>system</t>
         </is>
       </c>
       <c r="F28" s="5" t="n"/>
@@ -1509,12 +1499,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Microcontroller</t>
+          <t>DAC</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Teensy 4.1</t>
+          <t>Adafruit MCP4728 (product 4470)</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1526,7 +1516,7 @@
         </is>
       </c>
       <c r="F29" s="5" t="n">
-        <v>37.49</v>
+        <v>13</v>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
@@ -1535,12 +1525,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Antratek, incl. VAT</t>
+          <t>Opencircuit</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>https://www.antratek.de/teensy-4-1</t>
+          <t>https://opencircuit.shop/product/adafruit-mcp4728-quad-dac-with-eeprom</t>
         </is>
       </c>
       <c r="J29" s="5">
@@ -1556,12 +1546,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Pin headers for the Teensy</t>
+          <t>Carrier PCB</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2.54 mm male, 2 x 24</t>
+          <t>hardware/carrier, made at the makerspace</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1593,40 +1583,30 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DAC</t>
+          <t>Female header 1 x 24, 2.54 mm, 8.5 mm tall</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Adafruit MCP4728 (product 4470)</t>
+          <t>Teensy socket</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F31" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Opencircuit</t>
-        </is>
-      </c>
-      <c r="I31" s="7" t="inlineStr">
-        <is>
-          <t>https://opencircuit.shop/product/adafruit-mcp4728-quad-dac-with-eeprom</t>
-        </is>
-      </c>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>to check</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" s="5">
         <f>IF(F31="","",D31*F31*IF(E31="tower",$C$3,1))</f>
         <v/>
@@ -1640,16 +1620,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Carrier PCB</t>
+          <t>Female header 1 x 6, 2.54 mm</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>hardware/carrier, made at the makerspace</t>
+          <t>DAC socket</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1677,30 +1657,40 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Female header 1 x 24, 2.54 mm, 8.5 mm tall</t>
+          <t>PCB screw terminal 5-way, 5.08 mm</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Teensy socket</t>
+          <t>Phoenix Contact MKDS 1,5/5-5,08, 1715750</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="8" t="inlineStr">
-        <is>
-          <t>to check</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
+      <c r="F33" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>4-way 1715747 is EUR 2.26 at RS DE; 5-way similar</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>https://www.phoenixcontact.com/en-pc/products/pcb-terminal-block-mkds-15-5-508-1715750</t>
+        </is>
+      </c>
       <c r="J33" s="5">
         <f>IF(F33="","",D33*F33*IF(E33="tower",$C$3,1))</f>
         <v/>
@@ -1714,16 +1704,16 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Female header 1 x 6, 2.54 mm</t>
+          <t>Resistor 1 kOhm, 0.25 W, 1 %, axial</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>DAC socket</t>
+          <t>R1-R4</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1751,12 +1741,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PCB screw terminal 5-way, 5.08 mm</t>
+          <t>Resistor 1 MOhm, 0.25 W, 1 %, axial</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Phoenix Contact MKDS 1,5/5-5,08, 1715750</t>
+          <t>R5-R8</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1767,24 +1757,14 @@
           <t>system</t>
         </is>
       </c>
-      <c r="F35" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G35" s="9" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>4-way 1715747 is EUR 2.26 at RS DE; 5-way similar</t>
-        </is>
-      </c>
-      <c r="I35" s="7" t="inlineStr">
-        <is>
-          <t>https://www.phoenixcontact.com/en-pc/products/pcb-terminal-block-mkds-15-5-508-1715750</t>
-        </is>
-      </c>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>to check</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
       <c r="J35" s="5">
         <f>IF(F35="","",D35*F35*IF(E35="tower",$C$3,1))</f>
         <v/>
@@ -1798,12 +1778,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Resistor 1 kOhm, 0.25 W, 1 %, axial</t>
+          <t>Schottky diode</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>R1-R4</t>
+          <t>BAT85, DO-35 (D1-D4)</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1835,16 +1815,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Resistor 1 MOhm, 0.25 W, 1 %, axial</t>
+          <t>USB cable for the Teensy</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>R5-R8</t>
+          <t>micro-USB</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1867,21 +1847,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Control (once)</t>
+          <t>Safety &amp; harness (once)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Schottky diode</t>
+          <t>E-stop button + 1 NO contact block per 48 V supply + 24 AWG 2-wire cable</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>BAT85, DO-35 (D1-D4)</t>
+          <t>Stanford guide p. 13</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1904,17 +1884,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Control (once)</t>
+          <t>Safety &amp; harness (once)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>USB cable for the Teensy</t>
+          <t>Hip harness</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>micro-USB</t>
+          <t>Black Diamond climbing harness (Stanford)</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1946,12 +1926,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>E-stop button + 1 NO contact block per 48 V supply + 24 AWG 2-wire cable</t>
+          <t>Breakaway line</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Stanford guide p. 13</t>
+          <t>Berkley FireLine (Stanford guide p. 18)</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1983,12 +1963,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Hip harness</t>
+          <t>PLA filament</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Black Diamond climbing harness (Stanford)</t>
+          <t>1 reel, for all printed parts</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2020,12 +2000,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Breakaway line</t>
+          <t>Calibration weights</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Berkley FireLine (Stanford guide p. 18)</t>
+          <t>6, 8, 12 kg (thesis) - the lab may have them</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2049,104 +2029,30 @@
         <v/>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Safety &amp; harness (once)</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>PLA filament</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>1 reel, for all printed parts</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>system</t>
-        </is>
-      </c>
-      <c r="F43" s="5" t="n"/>
-      <c r="G43" s="8" t="inlineStr">
-        <is>
-          <t>to check</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" s="5">
-        <f>IF(F43="","",D43*F43*IF(E43="tower",$C$3,1))</f>
-        <v/>
-      </c>
-    </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Safety &amp; harness (once)</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Calibration weights</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>6, 8, 12 kg (thesis) - the lab may have them</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>system</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="n"/>
-      <c r="G44" s="8" t="inlineStr">
-        <is>
-          <t>to check</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" s="5">
-        <f>IF(F44="","",D44*F44*IF(E44="tower",$C$3,1))</f>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL (priced items)</t>
+        </is>
+      </c>
+      <c r="J44" s="10">
+        <f>SUM(J6:J42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Items still without a price</t>
+        </is>
+      </c>
+      <c r="J45">
+        <f>COUNTIF(G6:G42,"to check")</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL (priced items)</t>
-        </is>
-      </c>
-      <c r="J46" s="10">
-        <f>SUM(J6:J44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>Items still without a price</t>
-        </is>
-      </c>
-      <c r="J47">
-        <f>COUNTIF(G6:G44,"to check")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="I48" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>Note: mixes prices incl. and excl. VAT (see column H)</t>
         </is>
@@ -2156,20 +2062,18 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2197,7 +2101,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Not included: motor (maxon EC 90 flat 500267, Hall sensors built in), optional encoder (Renishaw RM22), aluminium frame (80x80 profiles).</t>
+          <t>Not included: motor (maxon EC 90 flat 500267, Hall sensors built in), optional encoder (Renishaw RM22), aluminium frame (80x80 profiles), 48 V supplies (Mean Well RSP-2000-48) and 24 V supplies (Mean Well RS-15-24): already in stock.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: carrier board pluggable module connectors (Phoenix MSTB 2,5 with flanges), board 154 x 96 mm
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parts-list.xlsx
+++ b/docs/parts-list.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1657,12 +1657,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PCB screw terminal 5-way, 5.08 mm</t>
+          <t>Board header, pluggable, 5-way, threaded flange</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Phoenix Contact MKDS 1,5/5-5,08, 1715750</t>
+          <t>Phoenix Contact MSTB 2,5/5-GF-5,08, 1776537</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1673,22 +1673,16 @@
           <t>system</t>
         </is>
       </c>
-      <c r="F33" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G33" s="9" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>4-way 1715747 is EUR 2.26 at RS DE; 5-way similar</t>
-        </is>
-      </c>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>to check</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>https://www.phoenixcontact.com/en-pc/products/pcb-terminal-block-mkds-15-5-508-1715750</t>
+          <t>https://www.phoenixcontact.com/en-us/products/pcb-header-mstb-25-5-gf-508-1776537</t>
         </is>
       </c>
       <c r="J33" s="5">
@@ -1704,12 +1698,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Resistor 1 kOhm, 0.25 W, 1 %, axial</t>
+          <t>Cable plug, 5-way, screw flange</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>R1-R4</t>
+          <t>Phoenix Contact MSTB 2,5/5-STF-5,08, 1778014</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1727,7 +1721,11 @@
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>https://www.phoenixcontact.com/en-us/products/pcb-plug-mstb-25-5-stf-508-1778014</t>
+        </is>
+      </c>
       <c r="J34" s="5">
         <f>IF(F34="","",D34*F34*IF(E34="tower",$C$3,1))</f>
         <v/>
@@ -1741,16 +1739,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Resistor 1 MOhm, 0.25 W, 1 %, axial</t>
+          <t>Coding profile (optional, keys each socket)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>R5-R8</t>
+          <t>Phoenix Contact CP-MSTB, 1734634 (pack of 100)</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1764,7 +1762,11 @@
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>https://www.phoenixcontact.com/en-us/products/coding-element-cp-mstb-1734634</t>
+        </is>
+      </c>
       <c r="J35" s="5">
         <f>IF(F35="","",D35*F35*IF(E35="tower",$C$3,1))</f>
         <v/>
@@ -1778,12 +1780,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Schottky diode</t>
+          <t>Resistor 1 kOhm, 0.25 W, 1 %, axial</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>BAT85, DO-35 (D1-D4)</t>
+          <t>R1-R4</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1815,16 +1817,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>USB cable for the Teensy</t>
+          <t>Resistor 1 MOhm, 0.25 W, 1 %, axial</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>micro-USB</t>
+          <t>R5-R8</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1847,21 +1849,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Safety &amp; harness (once)</t>
+          <t>Control (once)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>E-stop button + 1 NO contact block per 48 V supply + 24 AWG 2-wire cable</t>
+          <t>Schottky diode</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Stanford guide p. 13</t>
+          <t>BAT85, DO-35 (D1-D4)</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1884,17 +1886,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Safety &amp; harness (once)</t>
+          <t>Control (once)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Hip harness</t>
+          <t>USB cable for the Teensy</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Black Diamond climbing harness (Stanford)</t>
+          <t>micro-USB</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1926,12 +1928,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Breakaway line</t>
+          <t>E-stop button + 1 NO contact block per 48 V supply + 24 AWG 2-wire cable</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Berkley FireLine (Stanford guide p. 18)</t>
+          <t>Stanford guide p. 13</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1963,12 +1965,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PLA filament</t>
+          <t>Hip harness</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1 reel, for all printed parts</t>
+          <t>Black Diamond climbing harness (Stanford)</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2000,12 +2002,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Calibration weights</t>
+          <t>Breakaway line</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>6, 8, 12 kg (thesis) - the lab may have them</t>
+          <t>Berkley FireLine (Stanford guide p. 18)</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2029,30 +2031,104 @@
         <v/>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Safety &amp; harness (once)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>PLA filament</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1 reel, for all printed parts</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="n"/>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>to check</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" s="5">
+        <f>IF(F43="","",D43*F43*IF(E43="tower",$C$3,1))</f>
+        <v/>
+      </c>
+    </row>
     <row r="44">
-      <c r="I44" s="2" t="inlineStr">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Safety &amp; harness (once)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Calibration weights</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>6, 8, 12 kg (thesis) - the lab may have them</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="n"/>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>to check</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" s="5">
+        <f>IF(F44="","",D44*F44*IF(E44="tower",$C$3,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>TOTAL (priced items)</t>
         </is>
       </c>
-      <c r="J44" s="10">
-        <f>SUM(J6:J42)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="I45" t="inlineStr">
+      <c r="J46" s="10">
+        <f>SUM(J6:J44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="I47" t="inlineStr">
         <is>
           <t>Items still without a price</t>
         </is>
       </c>
-      <c r="J45">
-        <f>COUNTIF(G6:G42,"to check")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="I46" t="inlineStr">
+      <c r="J47">
+        <f>COUNTIF(G6:G44,"to check")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="I48" t="inlineStr">
         <is>
           <t>Note: mixes prices incl. and excl. VAT (see column H)</t>
         </is>
@@ -2074,6 +2150,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: parts list, header link removed (unverified)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/parts-list.xlsx
+++ b/docs/parts-list.xlsx
@@ -1679,12 +1679,12 @@
           <t>to check</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" s="7" t="inlineStr">
-        <is>
-          <t>https://www.phoenixcontact.com/en-us/products/pcb-header-mstb-25-5-gf-508-1776537</t>
-        </is>
-      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>order no. from the KiCad footprint description; search 1776537 at phoenixcontact.com</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
       <c r="J33" s="5">
         <f>IF(F33="","",D33*F33*IF(E33="tower",$C$3,1))</f>
         <v/>
@@ -2149,9 +2149,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>